<commit_message>
feat: búsqueda de sedes en vivo, «Generar comprobante» y tipografía del formato
- Sedes: filtra en el navegador mientras se escribe, sin acentos ni mayúsculas; sólo queda «Limpiar» con el estilo del admin y el sondeo trae el catálogo completo.
- Pagos: la tarjeta «Generar comprobante» aparece también en la pantalla de PAGO APROBADO, antes de «Corregir la resolución».
- Formato DEC: las celdas que llena SUIF van en Arial 8 (evento en negritas) y la X de las casillas en Arial sin negritas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/plantillas/formato-pago-uif.xlsx
+++ b/resources/plantillas/formato-pago-uif.xlsx
@@ -540,7 +540,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -577,10 +579,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -602,23 +604,23 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>

</xml_diff>